<commit_message>
plan: Ded Moroz earnings at flat 350 RUB/unit (all sizes + snegurochki)
Ded Moroz sheet in earnings plan: 350 RUB/unit for every model. Per-model
total units and profit potential + totals. Full stock 43320 units x350 =
15.2M potential; realistic season ~8000 units = 2.8M.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XzNBEf4vaaEHRqeR8ZkfFA
</commit_message>
<xml_diff>
--- a/outputs/plan/план_заработка_по_товарам_2026.xlsx
+++ b/outputs/plan/план_заработка_по_товарам_2026.xlsx
@@ -33,8 +33,8 @@
     <sheet name="MEDICUBE" sheetId="24" state="visible" r:id="rId24"/>
     <sheet name="VT COSMETICS" sheetId="25" state="visible" r:id="rId25"/>
     <sheet name="MASIL" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet name="ДЕДЫ МОРОЗЫ" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet name="ЭЛЕКТРОНИКА" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet name="ЭЛЕКТРОНИКА" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="ДЕДЫ МОРОЗЫ" sheetId="28" state="visible" r:id="rId28"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -44,7 +44,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -89,6 +89,11 @@
     <font>
       <b val="1"/>
       <color rgb="001F6E43"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F6E43"/>
+      <sz val="12"/>
     </font>
   </fonts>
   <fills count="5">
@@ -140,7 +145,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -166,6 +171,9 @@
     <xf numFmtId="3" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -4520,88 +4528,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="32" customWidth="1" min="1" max="1"/>
-    <col width="6" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="7" t="inlineStr">
-        <is>
-          <t>ДЕДЫ МОРОЗЫ — план заработка (сезон НГ)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>2025: продано 4642, прибыль 294к (маржа ~4%). Цель 2026 ~8000 шт. Рычаг прибыли — WB (комиссия ниже Ozon) + наборы.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="15" t="inlineStr">
-        <is>
-          <t>План продаж 2026, шт</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>8000</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="15" t="inlineStr">
-        <is>
-          <t>Ожидаемая маржа, % (цель)</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>12%</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="15" t="inlineStr">
-        <is>
-          <t>Ср.цена, ₽ (2025)</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>1460</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>ОЖИДАЕМЫЙ ЗАРАБОТОК 2026, ₽</t>
-        </is>
-      </c>
-      <c r="C7" s="16" t="n">
-        <v>1401600</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="13" t="inlineStr">
-        <is>
-          <t>NB: при марже 2025 (4%) заработок был бы ~470к. Цель 12% (через WB+наборы) → ~1,4 млн. Детальный план — в файле «дед_морозы_единый_план».</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -4887,6 +4813,710 @@
       </c>
       <c r="F13" s="18" t="n">
         <v>-166</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="21" t="inlineStr">
+        <is>
+          <t>ДЕДЫ МОРОЗЫ — план заработка (350 ₽/шт, любой размер + снегурочки)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Заработок/шт зафиксирован 350 ₽. Всего = склад + придёт (контейнер). Сезон НГ, продавать на 3 витринах, не докупать.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>Артикул WB</t>
+        </is>
+      </c>
+      <c r="B4" s="14" t="inlineStr">
+        <is>
+          <t>Наименование</t>
+        </is>
+      </c>
+      <c r="C4" s="14" t="inlineStr">
+        <is>
+          <t>Остаток склад</t>
+        </is>
+      </c>
+      <c r="D4" s="14" t="inlineStr">
+        <is>
+          <t>Придёт</t>
+        </is>
+      </c>
+      <c r="E4" s="14" t="inlineStr">
+        <is>
+          <t>ВСЕГО шт</t>
+        </is>
+      </c>
+      <c r="F4" s="14" t="inlineStr">
+        <is>
+          <t>Заработок/шт ₽</t>
+        </is>
+      </c>
+      <c r="G4" s="14" t="inlineStr">
+        <is>
+          <t>Потенциал заработка ₽</t>
+        </is>
+      </c>
+      <c r="H4" s="14" t="inlineStr">
+        <is>
+          <t>млн ₽</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="n">
+        <v>48905926</v>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Дед Мороз (№1) красный с подарком за спиной</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="n">
+        <v>2579</v>
+      </c>
+      <c r="D5" s="5" t="n">
+        <v>930</v>
+      </c>
+      <c r="E5" s="5" t="n">
+        <v>3509</v>
+      </c>
+      <c r="F5" s="5" t="n">
+        <v>350</v>
+      </c>
+      <c r="G5" s="9" t="n">
+        <v>1228150</v>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>1,23 млн</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="n">
+        <v>103431810</v>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Дед Мороз (№10) серый</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="n">
+        <v>1444</v>
+      </c>
+      <c r="D6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="5" t="n">
+        <v>1444</v>
+      </c>
+      <c r="F6" s="5" t="n">
+        <v>350</v>
+      </c>
+      <c r="G6" s="9" t="n">
+        <v>505400</v>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>0,51 млн</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="n">
+        <v>104590122</v>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Дед Мороз (№11) в клетку</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="n">
+        <v>5430</v>
+      </c>
+      <c r="D7" s="5" t="n">
+        <v>5070</v>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>10500</v>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>350</v>
+      </c>
+      <c r="G7" s="9" t="n">
+        <v>3675000</v>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>3,67 млн</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="n">
+        <v>555134309</v>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Дед Мороз (№11) 45см клетка</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="n">
+        <v>1920</v>
+      </c>
+      <c r="D8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="5" t="n">
+        <v>1920</v>
+      </c>
+      <c r="F8" s="5" t="n">
+        <v>350</v>
+      </c>
+      <c r="G8" s="9" t="n">
+        <v>672000</v>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>0,67 млн</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="n">
+        <v>555135716</v>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Дед Мороз (№11) 50см клетка</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="D9" s="5" t="n">
+        <v>672</v>
+      </c>
+      <c r="E9" s="5" t="n">
+        <v>702</v>
+      </c>
+      <c r="F9" s="5" t="n">
+        <v>350</v>
+      </c>
+      <c r="G9" s="9" t="n">
+        <v>245700</v>
+      </c>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>0,25 млн</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="n">
+        <v>555151552</v>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Дед Мороз (№11) 65см</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="5" t="n">
+        <v>156</v>
+      </c>
+      <c r="E10" s="5" t="n">
+        <v>156</v>
+      </c>
+      <c r="F10" s="5" t="n">
+        <v>350</v>
+      </c>
+      <c r="G10" s="9" t="n">
+        <v>54600</v>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>0,05 млн</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="n">
+        <v>555169767</v>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Дед Мороз (№11) 85см клетка</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="D11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="F11" s="5" t="n">
+        <v>350</v>
+      </c>
+      <c r="G11" s="9" t="n">
+        <v>1750</v>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>0,00 млн</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="n">
+        <v>103441912</v>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Дед Мороз (№12) белый лыжи белые боты</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="n">
+        <v>3904</v>
+      </c>
+      <c r="D12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="5" t="n">
+        <v>3904</v>
+      </c>
+      <c r="F12" s="5" t="n">
+        <v>350</v>
+      </c>
+      <c r="G12" s="9" t="n">
+        <v>1366400</v>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>1,37 млн</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="n">
+        <v>103442522</v>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Дед Мороз (№13) белый лыжи черные боты</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="n">
+        <v>996</v>
+      </c>
+      <c r="D13" s="5" t="n">
+        <v>210</v>
+      </c>
+      <c r="E13" s="5" t="n">
+        <v>1206</v>
+      </c>
+      <c r="F13" s="5" t="n">
+        <v>350</v>
+      </c>
+      <c r="G13" s="9" t="n">
+        <v>422100</v>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>0,42 млн</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="n">
+        <v>48906308</v>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Дед Мороз (№3) красный с мишкой</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="n">
+        <v>3506</v>
+      </c>
+      <c r="D14" s="5" t="n">
+        <v>1200</v>
+      </c>
+      <c r="E14" s="5" t="n">
+        <v>4706</v>
+      </c>
+      <c r="F14" s="5" t="n">
+        <v>350</v>
+      </c>
+      <c r="G14" s="9" t="n">
+        <v>1647100</v>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>1,65 млн</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="n">
+        <v>555204573</v>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Дед Мороз (№3) 45см с мишкой</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="n">
+        <v>1421</v>
+      </c>
+      <c r="D15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="5" t="n">
+        <v>1421</v>
+      </c>
+      <c r="F15" s="5" t="n">
+        <v>350</v>
+      </c>
+      <c r="G15" s="9" t="n">
+        <v>497350</v>
+      </c>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>0,50 млн</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="n">
+        <v>555208894</v>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Дед Мороз (№3) 50см с мишкой</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="D16" s="5" t="n">
+        <v>444</v>
+      </c>
+      <c r="E16" s="5" t="n">
+        <v>504</v>
+      </c>
+      <c r="F16" s="5" t="n">
+        <v>350</v>
+      </c>
+      <c r="G16" s="9" t="n">
+        <v>176400</v>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>0,18 млн</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="n">
+        <v>48906952</v>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Дед Мороз (№5) красный с подарком в руке</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="n">
+        <v>4431</v>
+      </c>
+      <c r="D17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" s="5" t="n">
+        <v>4431</v>
+      </c>
+      <c r="F17" s="5" t="n">
+        <v>350</v>
+      </c>
+      <c r="G17" s="9" t="n">
+        <v>1550850</v>
+      </c>
+      <c r="H17" s="5" t="inlineStr">
+        <is>
+          <t>1,55 млн</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="n">
+        <v>555212357</v>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Дед Мороз (№5) 45см с подарком</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="n">
+        <v>1188</v>
+      </c>
+      <c r="D18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" s="5" t="n">
+        <v>1188</v>
+      </c>
+      <c r="F18" s="5" t="n">
+        <v>350</v>
+      </c>
+      <c r="G18" s="9" t="n">
+        <v>415800</v>
+      </c>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>0,42 млн</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="n">
+        <v>555213580</v>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Дед Мороз (№5) 50см с подарком</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="n">
+        <v>200</v>
+      </c>
+      <c r="D19" s="5" t="n">
+        <v>576</v>
+      </c>
+      <c r="E19" s="5" t="n">
+        <v>776</v>
+      </c>
+      <c r="F19" s="5" t="n">
+        <v>350</v>
+      </c>
+      <c r="G19" s="9" t="n">
+        <v>271600</v>
+      </c>
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>0,27 млн</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="n">
+        <v>48908708</v>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Дед Мороз (№6) блестящий</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="n">
+        <v>1519</v>
+      </c>
+      <c r="D20" s="5" t="n">
+        <v>990</v>
+      </c>
+      <c r="E20" s="5" t="n">
+        <v>2509</v>
+      </c>
+      <c r="F20" s="5" t="n">
+        <v>350</v>
+      </c>
+      <c r="G20" s="9" t="n">
+        <v>878150</v>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>0,88 млн</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="n">
+        <v>103431353</v>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Дед Мороз (№9) красный рябь</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="n">
+        <v>1290</v>
+      </c>
+      <c r="D21" s="5" t="n">
+        <v>930</v>
+      </c>
+      <c r="E21" s="5" t="n">
+        <v>2220</v>
+      </c>
+      <c r="F21" s="5" t="n">
+        <v>350</v>
+      </c>
+      <c r="G21" s="9" t="n">
+        <v>777000</v>
+      </c>
+      <c r="H21" s="5" t="inlineStr">
+        <is>
+          <t>0,78 млн</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="n">
+        <v>190314124</v>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>СГ-Белая с узорами</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="n">
+        <v>717</v>
+      </c>
+      <c r="D22" s="5" t="n">
+        <v>780</v>
+      </c>
+      <c r="E22" s="5" t="n">
+        <v>1497</v>
+      </c>
+      <c r="F22" s="5" t="n">
+        <v>350</v>
+      </c>
+      <c r="G22" s="9" t="n">
+        <v>523950</v>
+      </c>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>0,52 млн</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="n">
+        <v>190314349</v>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>СГ-Красная</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="n">
+        <v>212</v>
+      </c>
+      <c r="D23" s="5" t="n">
+        <v>510</v>
+      </c>
+      <c r="E23" s="5" t="n">
+        <v>722</v>
+      </c>
+      <c r="F23" s="5" t="n">
+        <v>350</v>
+      </c>
+      <c r="G23" s="9" t="n">
+        <v>252700</v>
+      </c>
+      <c r="H23" s="5" t="inlineStr">
+        <is>
+          <t>0,25 млн</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="n"/>
+      <c r="B24" s="11" t="inlineStr">
+        <is>
+          <t>ИТОГО</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="n"/>
+      <c r="D24" s="5" t="n"/>
+      <c r="E24" s="22" t="n">
+        <v>43320</v>
+      </c>
+      <c r="F24" s="5" t="n"/>
+      <c r="G24" s="12" t="n">
+        <v>15162000</v>
+      </c>
+      <c r="H24" s="23" t="inlineStr">
+        <is>
+          <t>15,2 млн ₽</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="15" t="inlineStr">
+        <is>
+          <t>План продать за сезон 2026, шт</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="15" t="inlineStr">
+        <is>
+          <t>Заработок сезона (8000×350), ₽</t>
+        </is>
+      </c>
+      <c r="G27" s="16" t="n">
+        <v>2800000</v>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>2,80 млн ₽</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="13" t="inlineStr">
+        <is>
+          <t>NB: весь сток 43 320 шт × 350 = потенциал 15,2 млн ₽, но за сезон реально ~8 000 шт. Остальное — следующие сезоны или не докупать.</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>